<commit_message>
Rename i-Ready references to English and Math diagnostics
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A7tJMriTbrpMVpksL4pK5D
</commit_message>
<xml_diff>
--- a/summer-diagnostic-tracker-sample.xlsx
+++ b/summer-diagnostic-tracker-sample.xlsx
@@ -496,10 +496,10 @@
     <t xml:space="preserve">Students</t>
   </si>
   <si>
-    <t xml:space="preserve">ELA completed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ELA %</t>
+    <t xml:space="preserve">English completed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English %</t>
   </si>
   <si>
     <t xml:space="preserve">Math completed</t>
@@ -508,7 +508,7 @@
     <t xml:space="preserve">Math %</t>
   </si>
   <si>
-    <t xml:space="preserve">Avg ELA score</t>
+    <t xml:space="preserve">Avg English score</t>
   </si>
   <si>
     <t xml:space="preserve">Avg Math score</t>
@@ -520,7 +520,7 @@
     <t xml:space="preserve">Placement vs. grade</t>
   </si>
   <si>
-    <t xml:space="preserve">ELA students</t>
+    <t xml:space="preserve">English students</t>
   </si>
   <si>
     <t xml:space="preserve">Math students</t>
@@ -553,7 +553,7 @@
     <t xml:space="preserve">Group C</t>
   </si>
   <si>
-    <t xml:space="preserve">Placement is the overall i-Ready placement level entered from the diagnostic report. Scores and placements here are invented for the demo.</t>
+    <t xml:space="preserve">Placement is the overall placement level entered from the diagnostic report. Scores and placements here are invented for the demo.</t>
   </si>
   <si>
     <t xml:space="preserve">Students:</t>
@@ -565,16 +565,16 @@
     <t xml:space="preserve">Group</t>
   </si>
   <si>
-    <t xml:space="preserve">ELA Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ELA Score</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ELA Placement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ELA vs. Grade</t>
+    <t xml:space="preserve">English Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English Score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English Placement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English vs. Grade</t>
   </si>
   <si>
     <t xml:space="preserve">Math Status</t>

</xml_diff>